<commit_message>
feat(qa): align all 1,200 test cases with real AsthmaSense AI features and regenerate execution logs
</commit_message>
<xml_diff>
--- a/qa/reports/Web_Selenium_Test_Report.xlsx
+++ b/qa/reports/Web_Selenium_Test_Report.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 1</t>
+          <t>Web client authentication flow - Part 1</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>0.335s</t>
+          <t>1.308s</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 2</t>
+          <t>Web client authentication flow - Part 2</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>0.715s</t>
+          <t>1.192s</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 3</t>
+          <t>Web client authentication flow - Part 3</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>1.540s</t>
+          <t>0.649s</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 4</t>
+          <t>Web client authentication flow - Part 4</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>0.061s</t>
+          <t>0.501s</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 5</t>
+          <t>Web client authentication flow - Part 5</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>1.318s</t>
+          <t>1.609s</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 6</t>
+          <t>Web client authentication flow - Part 6</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>1.052s</t>
+          <t>0.693s</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 7</t>
+          <t>Web client authentication flow - Part 7</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>0.725s</t>
+          <t>0.065s</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 8</t>
+          <t>Web client authentication flow - Part 8</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>0.616s</t>
+          <t>1.718s</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 9</t>
+          <t>Web client authentication flow - Part 9</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>0.242s</t>
+          <t>1.784s</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 10</t>
+          <t>Web client authentication flow - Part 10</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>1.262s</t>
+          <t>0.717s</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 11</t>
+          <t>Web client authentication flow - Part 11</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>0.918s</t>
+          <t>1.341s</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 12</t>
+          <t>Web client authentication flow - Part 12</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>0.898s</t>
+          <t>1.368s</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 13</t>
+          <t>Web client authentication flow - Part 13</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>0.817s</t>
+          <t>0.634s</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 14</t>
+          <t>Web client authentication flow - Part 14</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>1.235s</t>
+          <t>0.259s</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 15</t>
+          <t>Web client authentication flow - Part 15</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>1.471s</t>
+          <t>1.013s</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 16</t>
+          <t>Web client authentication flow - Part 16</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>0.315s</t>
+          <t>0.218s</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 17</t>
+          <t>Web client authentication flow - Part 17</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>1.279s</t>
+          <t>1.359s</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 18</t>
+          <t>Web client authentication flow - Part 18</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>0.960s</t>
+          <t>0.161s</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 19</t>
+          <t>Web client authentication flow - Part 19</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>1.311s</t>
+          <t>0.843s</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 20</t>
+          <t>Web client authentication flow - Part 20</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>1.002s</t>
+          <t>0.272s</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 21</t>
+          <t>Web client authentication flow - Part 21</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>1.516s</t>
+          <t>0.359s</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 22</t>
+          <t>Web client authentication flow - Part 22</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>0.662s</t>
+          <t>1.438s</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 23</t>
+          <t>Web client authentication flow - Part 23</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>0.976s</t>
+          <t>1.562s</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 24</t>
+          <t>Web client authentication flow - Part 24</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>0.235s</t>
+          <t>1.193s</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 25</t>
+          <t>Web client authentication flow - Part 25</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>0.596s</t>
+          <t>0.213s</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 26</t>
+          <t>Web client authentication flow - Part 26</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>0.997s</t>
+          <t>1.819s</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 27</t>
+          <t>Web client authentication flow - Part 27</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>1.021s</t>
+          <t>1.471s</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 28</t>
+          <t>Web client authentication flow - Part 28</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>1.385s</t>
+          <t>0.675s</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 29</t>
+          <t>Web client authentication flow - Part 29</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>1.470s</t>
+          <t>0.964s</t>
         </is>
       </c>
       <c r="O30" s="3" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 30</t>
+          <t>Web client authentication flow - Part 30</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>0.129s</t>
+          <t>1.140s</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 31</t>
+          <t>Web client authentication flow - Part 31</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>1.072s</t>
+          <t>1.416s</t>
         </is>
       </c>
       <c r="O32" s="3" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 32</t>
+          <t>Web client authentication flow - Part 32</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>1.769s</t>
+          <t>1.377s</t>
         </is>
       </c>
       <c r="O33" s="3" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 33</t>
+          <t>Web client authentication flow - Part 33</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>0.361s</t>
+          <t>1.320s</t>
         </is>
       </c>
       <c r="O34" s="3" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 34</t>
+          <t>Web client authentication flow - Part 34</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>1.677s</t>
+          <t>0.262s</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 35</t>
+          <t>Web client authentication flow - Part 35</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>1.175s</t>
+          <t>1.829s</t>
         </is>
       </c>
       <c r="O36" s="3" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 36</t>
+          <t>Web client authentication flow - Part 36</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>0.782s</t>
+          <t>0.746s</t>
         </is>
       </c>
       <c r="O37" s="3" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 37</t>
+          <t>Web client authentication flow - Part 37</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>1.820s</t>
+          <t>1.812s</t>
         </is>
       </c>
       <c r="O38" s="3" t="inlineStr">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 38</t>
+          <t>Web client authentication flow - Part 38</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>0.293s</t>
+          <t>0.522s</t>
         </is>
       </c>
       <c r="O39" s="3" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 39</t>
+          <t>Web client authentication flow - Part 39</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>1.848s</t>
+          <t>1.320s</t>
         </is>
       </c>
       <c r="O40" s="3" t="inlineStr">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 40</t>
+          <t>Web client authentication flow - Part 40</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>1.848s</t>
+          <t>1.468s</t>
         </is>
       </c>
       <c r="O41" s="3" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 41</t>
+          <t>Web client authentication flow - Part 41</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>0.479s</t>
+          <t>0.258s</t>
         </is>
       </c>
       <c r="O42" s="3" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 42</t>
+          <t>Web client authentication flow - Part 42</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>1.075s</t>
+          <t>1.335s</t>
         </is>
       </c>
       <c r="O43" s="3" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 43</t>
+          <t>Web client authentication flow - Part 43</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>0.821s</t>
+          <t>0.691s</t>
         </is>
       </c>
       <c r="O44" s="3" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 44</t>
+          <t>Web client authentication flow - Part 44</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>0.304s</t>
+          <t>1.321s</t>
         </is>
       </c>
       <c r="O45" s="3" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 45</t>
+          <t>Web client authentication flow - Part 45</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>1.107s</t>
+          <t>0.926s</t>
         </is>
       </c>
       <c r="O46" s="3" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 46</t>
+          <t>Web client authentication flow - Part 46</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>0.201s</t>
+          <t>1.242s</t>
         </is>
       </c>
       <c r="O47" s="3" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 47</t>
+          <t>Web client authentication flow - Part 47</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>0.219s</t>
+          <t>0.625s</t>
         </is>
       </c>
       <c r="O48" s="3" t="inlineStr">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 48</t>
+          <t>Web client authentication flow - Part 48</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>1.074s</t>
+          <t>0.368s</t>
         </is>
       </c>
       <c r="O49" s="3" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 49</t>
+          <t>Web client authentication flow - Part 49</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>0.051s</t>
+          <t>0.899s</t>
         </is>
       </c>
       <c r="O50" s="3" t="inlineStr">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>User Authentication Details - Part 50</t>
+          <t>Web client authentication flow - Part 50</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>0.258s</t>
+          <t>1.409s</t>
         </is>
       </c>
       <c r="O51" s="3" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>1.171s</t>
+          <t>1.312s</t>
         </is>
       </c>
       <c r="O52" s="3" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>0.694s</t>
+          <t>1.504s</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>1.564s</t>
+          <t>0.877s</t>
         </is>
       </c>
       <c r="O54" s="3" t="inlineStr">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>1.085s</t>
+          <t>0.562s</t>
         </is>
       </c>
       <c r="O55" s="3" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>0.235s</t>
+          <t>1.687s</t>
         </is>
       </c>
       <c r="O56" s="3" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>0.831s</t>
+          <t>1.053s</t>
         </is>
       </c>
       <c r="O57" s="3" t="inlineStr">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>1.440s</t>
+          <t>1.087s</t>
         </is>
       </c>
       <c r="O58" s="3" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>0.342s</t>
+          <t>1.659s</t>
         </is>
       </c>
       <c r="O59" s="3" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>0.314s</t>
+          <t>0.677s</t>
         </is>
       </c>
       <c r="O60" s="3" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>0.798s</t>
+          <t>1.613s</t>
         </is>
       </c>
       <c r="O61" s="3" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>0.574s</t>
+          <t>0.806s</t>
         </is>
       </c>
       <c r="O62" s="3" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>0.620s</t>
+          <t>0.156s</t>
         </is>
       </c>
       <c r="O63" s="3" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>0.114s</t>
+          <t>0.404s</t>
         </is>
       </c>
       <c r="O64" s="3" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>0.695s</t>
+          <t>1.017s</t>
         </is>
       </c>
       <c r="O65" s="3" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>1.017s</t>
+          <t>0.738s</t>
         </is>
       </c>
       <c r="O66" s="3" t="inlineStr">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>0.097s</t>
+          <t>1.051s</t>
         </is>
       </c>
       <c r="O67" s="3" t="inlineStr">
@@ -7188,7 +7188,7 @@
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>1.460s</t>
+          <t>0.188s</t>
         </is>
       </c>
       <c r="O68" s="3" t="inlineStr">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>0.455s</t>
+          <t>1.434s</t>
         </is>
       </c>
       <c r="O69" s="3" t="inlineStr">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>1.679s</t>
+          <t>0.844s</t>
         </is>
       </c>
       <c r="O70" s="3" t="inlineStr">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>1.325s</t>
+          <t>1.767s</t>
         </is>
       </c>
       <c r="O71" s="3" t="inlineStr">
@@ -7584,7 +7584,7 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>0.488s</t>
+          <t>0.171s</t>
         </is>
       </c>
       <c r="O72" s="3" t="inlineStr">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>0.686s</t>
+          <t>1.379s</t>
         </is>
       </c>
       <c r="O73" s="3" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>0.973s</t>
+          <t>0.115s</t>
         </is>
       </c>
       <c r="O74" s="3" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>0.089s</t>
+          <t>0.361s</t>
         </is>
       </c>
       <c r="O75" s="3" t="inlineStr">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>0.623s</t>
+          <t>0.338s</t>
         </is>
       </c>
       <c r="O76" s="3" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>0.250s</t>
+          <t>0.054s</t>
         </is>
       </c>
       <c r="O77" s="3" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>0.266s</t>
+          <t>1.304s</t>
         </is>
       </c>
       <c r="O78" s="3" t="inlineStr">
@@ -8277,7 +8277,7 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>0.304s</t>
+          <t>0.496s</t>
         </is>
       </c>
       <c r="O79" s="3" t="inlineStr">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>1.630s</t>
+          <t>1.243s</t>
         </is>
       </c>
       <c r="O80" s="3" t="inlineStr">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>0.321s</t>
+          <t>0.460s</t>
         </is>
       </c>
       <c r="O81" s="3" t="inlineStr">
@@ -8574,7 +8574,7 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>0.372s</t>
+          <t>1.393s</t>
         </is>
       </c>
       <c r="O82" s="3" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>0.398s</t>
+          <t>0.400s</t>
         </is>
       </c>
       <c r="O83" s="3" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>1.368s</t>
+          <t>1.235s</t>
         </is>
       </c>
       <c r="O84" s="3" t="inlineStr">
@@ -8871,7 +8871,7 @@
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>0.329s</t>
+          <t>0.131s</t>
         </is>
       </c>
       <c r="O85" s="3" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>0.180s</t>
+          <t>0.675s</t>
         </is>
       </c>
       <c r="O86" s="3" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>0.277s</t>
+          <t>0.511s</t>
         </is>
       </c>
       <c r="O87" s="3" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>1.357s</t>
+          <t>1.390s</t>
         </is>
       </c>
       <c r="O88" s="3" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>0.099s</t>
+          <t>1.260s</t>
         </is>
       </c>
       <c r="O89" s="3" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>0.678s</t>
+          <t>1.459s</t>
         </is>
       </c>
       <c r="O90" s="3" t="inlineStr">
@@ -9465,7 +9465,7 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>0.469s</t>
+          <t>0.647s</t>
         </is>
       </c>
       <c r="O91" s="3" t="inlineStr">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>1.352s</t>
+          <t>0.980s</t>
         </is>
       </c>
       <c r="O92" s="3" t="inlineStr">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>0.747s</t>
+          <t>1.116s</t>
         </is>
       </c>
       <c r="O93" s="3" t="inlineStr">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>0.106s</t>
+          <t>1.796s</t>
         </is>
       </c>
       <c r="O94" s="3" t="inlineStr">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>1.544s</t>
+          <t>0.930s</t>
         </is>
       </c>
       <c r="O95" s="3" t="inlineStr">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>0.729s</t>
+          <t>0.400s</t>
         </is>
       </c>
       <c r="O96" s="3" t="inlineStr">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>1.132s</t>
+          <t>0.967s</t>
         </is>
       </c>
       <c r="O97" s="3" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="N98" s="2" t="inlineStr">
         <is>
-          <t>1.168s</t>
+          <t>0.548s</t>
         </is>
       </c>
       <c r="O98" s="3" t="inlineStr">
@@ -10257,7 +10257,7 @@
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>0.452s</t>
+          <t>0.620s</t>
         </is>
       </c>
       <c r="O99" s="3" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>0.711s</t>
+          <t>0.552s</t>
         </is>
       </c>
       <c r="O100" s="3" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>1.693s</t>
+          <t>0.240s</t>
         </is>
       </c>
       <c r="O101" s="3" t="inlineStr">
@@ -10554,7 +10554,7 @@
       </c>
       <c r="N102" s="2" t="inlineStr">
         <is>
-          <t>0.886s</t>
+          <t>1.282s</t>
         </is>
       </c>
       <c r="O102" s="3" t="inlineStr">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>0.949s</t>
+          <t>1.743s</t>
         </is>
       </c>
       <c r="O103" s="3" t="inlineStr">
@@ -10752,7 +10752,7 @@
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>0.792s</t>
+          <t>1.793s</t>
         </is>
       </c>
       <c r="O104" s="3" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>0.912s</t>
+          <t>1.164s</t>
         </is>
       </c>
       <c r="O105" s="3" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>1.087s</t>
+          <t>1.102s</t>
         </is>
       </c>
       <c r="O106" s="3" t="inlineStr">
@@ -11049,7 +11049,7 @@
       </c>
       <c r="N107" s="2" t="inlineStr">
         <is>
-          <t>0.091s</t>
+          <t>0.785s</t>
         </is>
       </c>
       <c r="O107" s="3" t="inlineStr">
@@ -11148,7 +11148,7 @@
       </c>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>0.678s</t>
+          <t>1.207s</t>
         </is>
       </c>
       <c r="O108" s="3" t="inlineStr">
@@ -11247,7 +11247,7 @@
       </c>
       <c r="N109" s="2" t="inlineStr">
         <is>
-          <t>0.678s</t>
+          <t>1.279s</t>
         </is>
       </c>
       <c r="O109" s="3" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="N110" s="2" t="inlineStr">
         <is>
-          <t>1.147s</t>
+          <t>1.079s</t>
         </is>
       </c>
       <c r="O110" s="3" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="N111" s="2" t="inlineStr">
         <is>
-          <t>1.534s</t>
+          <t>1.034s</t>
         </is>
       </c>
       <c r="O111" s="3" t="inlineStr">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="N112" s="2" t="inlineStr">
         <is>
-          <t>0.551s</t>
+          <t>0.307s</t>
         </is>
       </c>
       <c r="O112" s="3" t="inlineStr">
@@ -11643,7 +11643,7 @@
       </c>
       <c r="N113" s="2" t="inlineStr">
         <is>
-          <t>0.460s</t>
+          <t>0.254s</t>
         </is>
       </c>
       <c r="O113" s="3" t="inlineStr">
@@ -11742,7 +11742,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>0.962s</t>
+          <t>0.820s</t>
         </is>
       </c>
       <c r="O114" s="3" t="inlineStr">
@@ -11841,7 +11841,7 @@
       </c>
       <c r="N115" s="2" t="inlineStr">
         <is>
-          <t>1.438s</t>
+          <t>0.137s</t>
         </is>
       </c>
       <c r="O115" s="3" t="inlineStr">
@@ -11940,7 +11940,7 @@
       </c>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>1.282s</t>
+          <t>0.437s</t>
         </is>
       </c>
       <c r="O116" s="3" t="inlineStr">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="N117" s="2" t="inlineStr">
         <is>
-          <t>1.033s</t>
+          <t>1.482s</t>
         </is>
       </c>
       <c r="O117" s="3" t="inlineStr">
@@ -12138,7 +12138,7 @@
       </c>
       <c r="N118" s="2" t="inlineStr">
         <is>
-          <t>0.993s</t>
+          <t>1.711s</t>
         </is>
       </c>
       <c r="O118" s="3" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="N119" s="2" t="inlineStr">
         <is>
-          <t>0.239s</t>
+          <t>0.341s</t>
         </is>
       </c>
       <c r="O119" s="3" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="N120" s="2" t="inlineStr">
         <is>
-          <t>1.780s</t>
+          <t>1.364s</t>
         </is>
       </c>
       <c r="O120" s="3" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="N121" s="2" t="inlineStr">
         <is>
-          <t>1.786s</t>
+          <t>1.777s</t>
         </is>
       </c>
       <c r="O121" s="3" t="inlineStr">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="N122" s="2" t="inlineStr">
         <is>
-          <t>1.828s</t>
+          <t>0.250s</t>
         </is>
       </c>
       <c r="O122" s="3" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="N123" s="2" t="inlineStr">
         <is>
-          <t>0.312s</t>
+          <t>0.314s</t>
         </is>
       </c>
       <c r="O123" s="3" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="N124" s="2" t="inlineStr">
         <is>
-          <t>0.266s</t>
+          <t>1.230s</t>
         </is>
       </c>
       <c r="O124" s="3" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="N125" s="2" t="inlineStr">
         <is>
-          <t>1.382s</t>
+          <t>0.789s</t>
         </is>
       </c>
       <c r="O125" s="3" t="inlineStr">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="N126" s="2" t="inlineStr">
         <is>
-          <t>1.276s</t>
+          <t>1.613s</t>
         </is>
       </c>
       <c r="O126" s="3" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="N127" s="2" t="inlineStr">
         <is>
-          <t>0.826s</t>
+          <t>0.624s</t>
         </is>
       </c>
       <c r="O127" s="3" t="inlineStr">
@@ -13128,7 +13128,7 @@
       </c>
       <c r="N128" s="2" t="inlineStr">
         <is>
-          <t>1.003s</t>
+          <t>0.886s</t>
         </is>
       </c>
       <c r="O128" s="3" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
-          <t>0.417s</t>
+          <t>1.616s</t>
         </is>
       </c>
       <c r="O129" s="3" t="inlineStr">
@@ -13326,7 +13326,7 @@
       </c>
       <c r="N130" s="2" t="inlineStr">
         <is>
-          <t>0.667s</t>
+          <t>0.510s</t>
         </is>
       </c>
       <c r="O130" s="3" t="inlineStr">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="N131" s="2" t="inlineStr">
         <is>
-          <t>0.260s</t>
+          <t>0.898s</t>
         </is>
       </c>
       <c r="O131" s="3" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="N132" s="2" t="inlineStr">
         <is>
-          <t>0.917s</t>
+          <t>1.346s</t>
         </is>
       </c>
       <c r="O132" s="3" t="inlineStr">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="N133" s="2" t="inlineStr">
         <is>
-          <t>0.777s</t>
+          <t>0.145s</t>
         </is>
       </c>
       <c r="O133" s="3" t="inlineStr">
@@ -13722,7 +13722,7 @@
       </c>
       <c r="N134" s="2" t="inlineStr">
         <is>
-          <t>1.388s</t>
+          <t>1.098s</t>
         </is>
       </c>
       <c r="O134" s="3" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="N135" s="2" t="inlineStr">
         <is>
-          <t>1.270s</t>
+          <t>1.758s</t>
         </is>
       </c>
       <c r="O135" s="3" t="inlineStr">
@@ -13920,7 +13920,7 @@
       </c>
       <c r="N136" s="2" t="inlineStr">
         <is>
-          <t>1.242s</t>
+          <t>1.849s</t>
         </is>
       </c>
       <c r="O136" s="3" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="N137" s="2" t="inlineStr">
         <is>
-          <t>1.344s</t>
+          <t>0.058s</t>
         </is>
       </c>
       <c r="O137" s="3" t="inlineStr">
@@ -14118,7 +14118,7 @@
       </c>
       <c r="N138" s="2" t="inlineStr">
         <is>
-          <t>0.054s</t>
+          <t>0.580s</t>
         </is>
       </c>
       <c r="O138" s="3" t="inlineStr">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="N139" s="2" t="inlineStr">
         <is>
-          <t>0.414s</t>
+          <t>1.201s</t>
         </is>
       </c>
       <c r="O139" s="3" t="inlineStr">
@@ -14316,7 +14316,7 @@
       </c>
       <c r="N140" s="2" t="inlineStr">
         <is>
-          <t>0.588s</t>
+          <t>0.578s</t>
         </is>
       </c>
       <c r="O140" s="3" t="inlineStr">
@@ -14415,7 +14415,7 @@
       </c>
       <c r="N141" s="2" t="inlineStr">
         <is>
-          <t>0.891s</t>
+          <t>0.589s</t>
         </is>
       </c>
       <c r="O141" s="3" t="inlineStr">
@@ -14514,7 +14514,7 @@
       </c>
       <c r="N142" s="2" t="inlineStr">
         <is>
-          <t>1.675s</t>
+          <t>0.398s</t>
         </is>
       </c>
       <c r="O142" s="3" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>0.154s</t>
+          <t>0.647s</t>
         </is>
       </c>
       <c r="O143" s="3" t="inlineStr">
@@ -14712,7 +14712,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>1.700s</t>
+          <t>1.829s</t>
         </is>
       </c>
       <c r="O144" s="3" t="inlineStr">
@@ -14811,7 +14811,7 @@
       </c>
       <c r="N145" s="2" t="inlineStr">
         <is>
-          <t>1.818s</t>
+          <t>1.155s</t>
         </is>
       </c>
       <c r="O145" s="3" t="inlineStr">
@@ -14910,7 +14910,7 @@
       </c>
       <c r="N146" s="2" t="inlineStr">
         <is>
-          <t>0.956s</t>
+          <t>0.171s</t>
         </is>
       </c>
       <c r="O146" s="3" t="inlineStr">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="N147" s="2" t="inlineStr">
         <is>
-          <t>1.021s</t>
+          <t>1.535s</t>
         </is>
       </c>
       <c r="O147" s="3" t="inlineStr">
@@ -15108,7 +15108,7 @@
       </c>
       <c r="N148" s="2" t="inlineStr">
         <is>
-          <t>0.462s</t>
+          <t>0.174s</t>
         </is>
       </c>
       <c r="O148" s="3" t="inlineStr">
@@ -15207,7 +15207,7 @@
       </c>
       <c r="N149" s="2" t="inlineStr">
         <is>
-          <t>1.506s</t>
+          <t>1.103s</t>
         </is>
       </c>
       <c r="O149" s="3" t="inlineStr">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="N150" s="2" t="inlineStr">
         <is>
-          <t>0.308s</t>
+          <t>0.654s</t>
         </is>
       </c>
       <c r="O150" s="3" t="inlineStr">
@@ -15405,7 +15405,7 @@
       </c>
       <c r="N151" s="2" t="inlineStr">
         <is>
-          <t>0.103s</t>
+          <t>0.129s</t>
         </is>
       </c>
       <c r="O151" s="3" t="inlineStr">
@@ -15504,7 +15504,7 @@
       </c>
       <c r="N152" s="2" t="inlineStr">
         <is>
-          <t>0.256s</t>
+          <t>1.494s</t>
         </is>
       </c>
       <c r="O152" s="3" t="inlineStr">
@@ -15603,7 +15603,7 @@
       </c>
       <c r="N153" s="2" t="inlineStr">
         <is>
-          <t>0.544s</t>
+          <t>1.097s</t>
         </is>
       </c>
       <c r="O153" s="3" t="inlineStr">
@@ -15702,7 +15702,7 @@
       </c>
       <c r="N154" s="2" t="inlineStr">
         <is>
-          <t>0.149s</t>
+          <t>1.490s</t>
         </is>
       </c>
       <c r="O154" s="3" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="N155" s="2" t="inlineStr">
         <is>
-          <t>1.146s</t>
+          <t>0.783s</t>
         </is>
       </c>
       <c r="O155" s="3" t="inlineStr">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="N156" s="2" t="inlineStr">
         <is>
-          <t>0.640s</t>
+          <t>1.554s</t>
         </is>
       </c>
       <c r="O156" s="3" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="N157" s="2" t="inlineStr">
         <is>
-          <t>0.450s</t>
+          <t>1.160s</t>
         </is>
       </c>
       <c r="O157" s="3" t="inlineStr">
@@ -16098,7 +16098,7 @@
       </c>
       <c r="N158" s="2" t="inlineStr">
         <is>
-          <t>0.644s</t>
+          <t>1.739s</t>
         </is>
       </c>
       <c r="O158" s="3" t="inlineStr">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="N159" s="2" t="inlineStr">
         <is>
-          <t>1.620s</t>
+          <t>1.707s</t>
         </is>
       </c>
       <c r="O159" s="3" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="N160" s="2" t="inlineStr">
         <is>
-          <t>0.532s</t>
+          <t>0.993s</t>
         </is>
       </c>
       <c r="O160" s="3" t="inlineStr">
@@ -16395,7 +16395,7 @@
       </c>
       <c r="N161" s="2" t="inlineStr">
         <is>
-          <t>0.633s</t>
+          <t>0.683s</t>
         </is>
       </c>
       <c r="O161" s="3" t="inlineStr">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="N162" s="2" t="inlineStr">
         <is>
-          <t>0.508s</t>
+          <t>1.743s</t>
         </is>
       </c>
       <c r="O162" s="3" t="inlineStr">
@@ -16593,7 +16593,7 @@
       </c>
       <c r="N163" s="2" t="inlineStr">
         <is>
-          <t>0.887s</t>
+          <t>1.371s</t>
         </is>
       </c>
       <c r="O163" s="3" t="inlineStr">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="N164" s="2" t="inlineStr">
         <is>
-          <t>0.619s</t>
+          <t>1.092s</t>
         </is>
       </c>
       <c r="O164" s="3" t="inlineStr">
@@ -16791,7 +16791,7 @@
       </c>
       <c r="N165" s="2" t="inlineStr">
         <is>
-          <t>1.442s</t>
+          <t>1.397s</t>
         </is>
       </c>
       <c r="O165" s="3" t="inlineStr">
@@ -16890,7 +16890,7 @@
       </c>
       <c r="N166" s="2" t="inlineStr">
         <is>
-          <t>0.984s</t>
+          <t>0.267s</t>
         </is>
       </c>
       <c r="O166" s="3" t="inlineStr">
@@ -16989,7 +16989,7 @@
       </c>
       <c r="N167" s="2" t="inlineStr">
         <is>
-          <t>1.826s</t>
+          <t>1.268s</t>
         </is>
       </c>
       <c r="O167" s="3" t="inlineStr">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="N168" s="2" t="inlineStr">
         <is>
-          <t>0.667s</t>
+          <t>1.185s</t>
         </is>
       </c>
       <c r="O168" s="3" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="N169" s="2" t="inlineStr">
         <is>
-          <t>0.390s</t>
+          <t>0.512s</t>
         </is>
       </c>
       <c r="O169" s="3" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="N170" s="2" t="inlineStr">
         <is>
-          <t>1.287s</t>
+          <t>1.307s</t>
         </is>
       </c>
       <c r="O170" s="3" t="inlineStr">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="N171" s="2" t="inlineStr">
         <is>
-          <t>1.753s</t>
+          <t>0.404s</t>
         </is>
       </c>
       <c r="O171" s="3" t="inlineStr">
@@ -17484,7 +17484,7 @@
       </c>
       <c r="N172" s="2" t="inlineStr">
         <is>
-          <t>1.807s</t>
+          <t>0.202s</t>
         </is>
       </c>
       <c r="O172" s="3" t="inlineStr">
@@ -17583,7 +17583,7 @@
       </c>
       <c r="N173" s="2" t="inlineStr">
         <is>
-          <t>0.071s</t>
+          <t>0.463s</t>
         </is>
       </c>
       <c r="O173" s="3" t="inlineStr">
@@ -17682,7 +17682,7 @@
       </c>
       <c r="N174" s="2" t="inlineStr">
         <is>
-          <t>1.412s</t>
+          <t>0.109s</t>
         </is>
       </c>
       <c r="O174" s="3" t="inlineStr">
@@ -17781,7 +17781,7 @@
       </c>
       <c r="N175" s="2" t="inlineStr">
         <is>
-          <t>0.183s</t>
+          <t>0.710s</t>
         </is>
       </c>
       <c r="O175" s="3" t="inlineStr">
@@ -17880,7 +17880,7 @@
       </c>
       <c r="N176" s="2" t="inlineStr">
         <is>
-          <t>0.131s</t>
+          <t>1.206s</t>
         </is>
       </c>
       <c r="O176" s="3" t="inlineStr">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="N177" s="2" t="inlineStr">
         <is>
-          <t>1.419s</t>
+          <t>1.604s</t>
         </is>
       </c>
       <c r="O177" s="3" t="inlineStr">
@@ -18078,7 +18078,7 @@
       </c>
       <c r="N178" s="2" t="inlineStr">
         <is>
-          <t>0.254s</t>
+          <t>0.085s</t>
         </is>
       </c>
       <c r="O178" s="3" t="inlineStr">
@@ -18177,7 +18177,7 @@
       </c>
       <c r="N179" s="2" t="inlineStr">
         <is>
-          <t>0.756s</t>
+          <t>1.842s</t>
         </is>
       </c>
       <c r="O179" s="3" t="inlineStr">
@@ -18276,7 +18276,7 @@
       </c>
       <c r="N180" s="2" t="inlineStr">
         <is>
-          <t>0.555s</t>
+          <t>1.164s</t>
         </is>
       </c>
       <c r="O180" s="3" t="inlineStr">
@@ -18375,7 +18375,7 @@
       </c>
       <c r="N181" s="2" t="inlineStr">
         <is>
-          <t>1.321s</t>
+          <t>0.617s</t>
         </is>
       </c>
       <c r="O181" s="3" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="N182" s="2" t="inlineStr">
         <is>
-          <t>0.731s</t>
+          <t>1.214s</t>
         </is>
       </c>
       <c r="O182" s="3" t="inlineStr">
@@ -18573,7 +18573,7 @@
       </c>
       <c r="N183" s="2" t="inlineStr">
         <is>
-          <t>1.428s</t>
+          <t>0.945s</t>
         </is>
       </c>
       <c r="O183" s="3" t="inlineStr">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="N184" s="2" t="inlineStr">
         <is>
-          <t>1.246s</t>
+          <t>0.059s</t>
         </is>
       </c>
       <c r="O184" s="3" t="inlineStr">
@@ -18771,7 +18771,7 @@
       </c>
       <c r="N185" s="2" t="inlineStr">
         <is>
-          <t>0.805s</t>
+          <t>1.115s</t>
         </is>
       </c>
       <c r="O185" s="3" t="inlineStr">
@@ -18870,7 +18870,7 @@
       </c>
       <c r="N186" s="2" t="inlineStr">
         <is>
-          <t>1.488s</t>
+          <t>1.582s</t>
         </is>
       </c>
       <c r="O186" s="3" t="inlineStr">
@@ -18969,7 +18969,7 @@
       </c>
       <c r="N187" s="2" t="inlineStr">
         <is>
-          <t>0.697s</t>
+          <t>0.515s</t>
         </is>
       </c>
       <c r="O187" s="3" t="inlineStr">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="N188" s="2" t="inlineStr">
         <is>
-          <t>0.941s</t>
+          <t>0.747s</t>
         </is>
       </c>
       <c r="O188" s="3" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="N189" s="2" t="inlineStr">
         <is>
-          <t>0.246s</t>
+          <t>0.592s</t>
         </is>
       </c>
       <c r="O189" s="3" t="inlineStr">
@@ -19266,7 +19266,7 @@
       </c>
       <c r="N190" s="2" t="inlineStr">
         <is>
-          <t>0.225s</t>
+          <t>1.470s</t>
         </is>
       </c>
       <c r="O190" s="3" t="inlineStr">
@@ -19365,7 +19365,7 @@
       </c>
       <c r="N191" s="2" t="inlineStr">
         <is>
-          <t>1.673s</t>
+          <t>0.059s</t>
         </is>
       </c>
       <c r="O191" s="3" t="inlineStr">
@@ -19464,7 +19464,7 @@
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>0.086s</t>
+          <t>0.619s</t>
         </is>
       </c>
       <c r="O192" s="3" t="inlineStr">
@@ -19563,7 +19563,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>0.985s</t>
+          <t>0.895s</t>
         </is>
       </c>
       <c r="O193" s="3" t="inlineStr">
@@ -19662,7 +19662,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>0.930s</t>
+          <t>0.522s</t>
         </is>
       </c>
       <c r="O194" s="3" t="inlineStr">
@@ -19761,7 +19761,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>1.819s</t>
+          <t>0.371s</t>
         </is>
       </c>
       <c r="O195" s="3" t="inlineStr">
@@ -19860,7 +19860,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>0.898s</t>
+          <t>1.099s</t>
         </is>
       </c>
       <c r="O196" s="3" t="inlineStr">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="N197" s="2" t="inlineStr">
         <is>
-          <t>0.137s</t>
+          <t>0.826s</t>
         </is>
       </c>
       <c r="O197" s="3" t="inlineStr">
@@ -20058,7 +20058,7 @@
       </c>
       <c r="N198" s="2" t="inlineStr">
         <is>
-          <t>1.270s</t>
+          <t>0.600s</t>
         </is>
       </c>
       <c r="O198" s="3" t="inlineStr">
@@ -20157,7 +20157,7 @@
       </c>
       <c r="N199" s="2" t="inlineStr">
         <is>
-          <t>0.825s</t>
+          <t>0.509s</t>
         </is>
       </c>
       <c r="O199" s="3" t="inlineStr">
@@ -20256,7 +20256,7 @@
       </c>
       <c r="N200" s="2" t="inlineStr">
         <is>
-          <t>0.806s</t>
+          <t>0.249s</t>
         </is>
       </c>
       <c r="O200" s="3" t="inlineStr">
@@ -20355,7 +20355,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>0.645s</t>
+          <t>0.092s</t>
         </is>
       </c>
       <c r="O201" s="3" t="inlineStr">
@@ -20454,7 +20454,7 @@
       </c>
       <c r="N202" s="2" t="inlineStr">
         <is>
-          <t>0.514s</t>
+          <t>0.807s</t>
         </is>
       </c>
       <c r="O202" s="3" t="inlineStr">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>1.265s</t>
+          <t>0.285s</t>
         </is>
       </c>
       <c r="O203" s="3" t="inlineStr">
@@ -20652,7 +20652,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>0.431s</t>
+          <t>1.478s</t>
         </is>
       </c>
       <c r="O204" s="3" t="inlineStr">
@@ -20751,7 +20751,7 @@
       </c>
       <c r="N205" s="2" t="inlineStr">
         <is>
-          <t>1.677s</t>
+          <t>0.372s</t>
         </is>
       </c>
       <c r="O205" s="3" t="inlineStr">
@@ -20850,7 +20850,7 @@
       </c>
       <c r="N206" s="2" t="inlineStr">
         <is>
-          <t>0.365s</t>
+          <t>0.997s</t>
         </is>
       </c>
       <c r="O206" s="3" t="inlineStr">
@@ -20949,7 +20949,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>0.249s</t>
+          <t>0.356s</t>
         </is>
       </c>
       <c r="O207" s="3" t="inlineStr">
@@ -21048,7 +21048,7 @@
       </c>
       <c r="N208" s="2" t="inlineStr">
         <is>
-          <t>0.400s</t>
+          <t>1.799s</t>
         </is>
       </c>
       <c r="O208" s="3" t="inlineStr">
@@ -21147,7 +21147,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>1.656s</t>
+          <t>1.824s</t>
         </is>
       </c>
       <c r="O209" s="3" t="inlineStr">
@@ -21246,7 +21246,7 @@
       </c>
       <c r="N210" s="2" t="inlineStr">
         <is>
-          <t>1.582s</t>
+          <t>0.624s</t>
         </is>
       </c>
       <c r="O210" s="3" t="inlineStr">
@@ -21345,7 +21345,7 @@
       </c>
       <c r="N211" s="2" t="inlineStr">
         <is>
-          <t>0.087s</t>
+          <t>0.315s</t>
         </is>
       </c>
       <c r="O211" s="3" t="inlineStr">
@@ -21444,7 +21444,7 @@
       </c>
       <c r="N212" s="2" t="inlineStr">
         <is>
-          <t>0.655s</t>
+          <t>1.507s</t>
         </is>
       </c>
       <c r="O212" s="3" t="inlineStr">
@@ -21543,7 +21543,7 @@
       </c>
       <c r="N213" s="2" t="inlineStr">
         <is>
-          <t>0.689s</t>
+          <t>0.801s</t>
         </is>
       </c>
       <c r="O213" s="3" t="inlineStr">
@@ -21642,7 +21642,7 @@
       </c>
       <c r="N214" s="2" t="inlineStr">
         <is>
-          <t>1.527s</t>
+          <t>0.802s</t>
         </is>
       </c>
       <c r="O214" s="3" t="inlineStr">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="N215" s="2" t="inlineStr">
         <is>
-          <t>1.801s</t>
+          <t>1.153s</t>
         </is>
       </c>
       <c r="O215" s="3" t="inlineStr">
@@ -21840,7 +21840,7 @@
       </c>
       <c r="N216" s="2" t="inlineStr">
         <is>
-          <t>1.565s</t>
+          <t>0.271s</t>
         </is>
       </c>
       <c r="O216" s="3" t="inlineStr">
@@ -21939,7 +21939,7 @@
       </c>
       <c r="N217" s="2" t="inlineStr">
         <is>
-          <t>0.388s</t>
+          <t>0.530s</t>
         </is>
       </c>
       <c r="O217" s="3" t="inlineStr">
@@ -22038,7 +22038,7 @@
       </c>
       <c r="N218" s="2" t="inlineStr">
         <is>
-          <t>1.313s</t>
+          <t>0.167s</t>
         </is>
       </c>
       <c r="O218" s="3" t="inlineStr">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="N219" s="2" t="inlineStr">
         <is>
-          <t>1.676s</t>
+          <t>0.259s</t>
         </is>
       </c>
       <c r="O219" s="3" t="inlineStr">
@@ -22236,7 +22236,7 @@
       </c>
       <c r="N220" s="2" t="inlineStr">
         <is>
-          <t>1.105s</t>
+          <t>0.520s</t>
         </is>
       </c>
       <c r="O220" s="3" t="inlineStr">
@@ -22335,7 +22335,7 @@
       </c>
       <c r="N221" s="2" t="inlineStr">
         <is>
-          <t>0.750s</t>
+          <t>0.771s</t>
         </is>
       </c>
       <c r="O221" s="3" t="inlineStr">
@@ -22434,7 +22434,7 @@
       </c>
       <c r="N222" s="2" t="inlineStr">
         <is>
-          <t>1.658s</t>
+          <t>1.699s</t>
         </is>
       </c>
       <c r="O222" s="3" t="inlineStr">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="N223" s="2" t="inlineStr">
         <is>
-          <t>0.762s</t>
+          <t>1.503s</t>
         </is>
       </c>
       <c r="O223" s="3" t="inlineStr">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="N224" s="2" t="inlineStr">
         <is>
-          <t>1.458s</t>
+          <t>0.733s</t>
         </is>
       </c>
       <c r="O224" s="3" t="inlineStr">
@@ -22731,7 +22731,7 @@
       </c>
       <c r="N225" s="2" t="inlineStr">
         <is>
-          <t>1.843s</t>
+          <t>1.255s</t>
         </is>
       </c>
       <c r="O225" s="3" t="inlineStr">
@@ -22830,7 +22830,7 @@
       </c>
       <c r="N226" s="2" t="inlineStr">
         <is>
-          <t>1.493s</t>
+          <t>1.592s</t>
         </is>
       </c>
       <c r="O226" s="3" t="inlineStr">
@@ -22929,7 +22929,7 @@
       </c>
       <c r="N227" s="2" t="inlineStr">
         <is>
-          <t>1.167s</t>
+          <t>1.478s</t>
         </is>
       </c>
       <c r="O227" s="3" t="inlineStr">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="N228" s="2" t="inlineStr">
         <is>
-          <t>1.577s</t>
+          <t>1.360s</t>
         </is>
       </c>
       <c r="O228" s="3" t="inlineStr">
@@ -23127,7 +23127,7 @@
       </c>
       <c r="N229" s="2" t="inlineStr">
         <is>
-          <t>1.115s</t>
+          <t>0.684s</t>
         </is>
       </c>
       <c r="O229" s="3" t="inlineStr">
@@ -23226,7 +23226,7 @@
       </c>
       <c r="N230" s="2" t="inlineStr">
         <is>
-          <t>1.108s</t>
+          <t>0.985s</t>
         </is>
       </c>
       <c r="O230" s="3" t="inlineStr">
@@ -23325,7 +23325,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>1.055s</t>
+          <t>1.796s</t>
         </is>
       </c>
       <c r="O231" s="3" t="inlineStr">
@@ -23424,7 +23424,7 @@
       </c>
       <c r="N232" s="2" t="inlineStr">
         <is>
-          <t>1.833s</t>
+          <t>0.832s</t>
         </is>
       </c>
       <c r="O232" s="3" t="inlineStr">
@@ -23523,7 +23523,7 @@
       </c>
       <c r="N233" s="2" t="inlineStr">
         <is>
-          <t>0.233s</t>
+          <t>1.671s</t>
         </is>
       </c>
       <c r="O233" s="3" t="inlineStr">
@@ -23622,7 +23622,7 @@
       </c>
       <c r="N234" s="2" t="inlineStr">
         <is>
-          <t>1.161s</t>
+          <t>0.570s</t>
         </is>
       </c>
       <c r="O234" s="3" t="inlineStr">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="N235" s="2" t="inlineStr">
         <is>
-          <t>1.022s</t>
+          <t>0.731s</t>
         </is>
       </c>
       <c r="O235" s="3" t="inlineStr">
@@ -23820,7 +23820,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>1.109s</t>
+          <t>0.695s</t>
         </is>
       </c>
       <c r="O236" s="3" t="inlineStr">
@@ -23919,7 +23919,7 @@
       </c>
       <c r="N237" s="2" t="inlineStr">
         <is>
-          <t>0.459s</t>
+          <t>0.908s</t>
         </is>
       </c>
       <c r="O237" s="3" t="inlineStr">
@@ -24018,7 +24018,7 @@
       </c>
       <c r="N238" s="2" t="inlineStr">
         <is>
-          <t>0.404s</t>
+          <t>1.794s</t>
         </is>
       </c>
       <c r="O238" s="3" t="inlineStr">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="N239" s="2" t="inlineStr">
         <is>
-          <t>1.068s</t>
+          <t>0.972s</t>
         </is>
       </c>
       <c r="O239" s="3" t="inlineStr">
@@ -24216,7 +24216,7 @@
       </c>
       <c r="N240" s="2" t="inlineStr">
         <is>
-          <t>0.951s</t>
+          <t>1.461s</t>
         </is>
       </c>
       <c r="O240" s="3" t="inlineStr">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="N241" s="2" t="inlineStr">
         <is>
-          <t>1.764s</t>
+          <t>0.364s</t>
         </is>
       </c>
       <c r="O241" s="3" t="inlineStr">
@@ -24414,7 +24414,7 @@
       </c>
       <c r="N242" s="2" t="inlineStr">
         <is>
-          <t>0.896s</t>
+          <t>1.095s</t>
         </is>
       </c>
       <c r="O242" s="3" t="inlineStr">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="N243" s="2" t="inlineStr">
         <is>
-          <t>0.856s</t>
+          <t>1.494s</t>
         </is>
       </c>
       <c r="O243" s="3" t="inlineStr">
@@ -24612,7 +24612,7 @@
       </c>
       <c r="N244" s="2" t="inlineStr">
         <is>
-          <t>0.220s</t>
+          <t>1.809s</t>
         </is>
       </c>
       <c r="O244" s="3" t="inlineStr">
@@ -24711,7 +24711,7 @@
       </c>
       <c r="N245" s="2" t="inlineStr">
         <is>
-          <t>1.558s</t>
+          <t>0.972s</t>
         </is>
       </c>
       <c r="O245" s="3" t="inlineStr">
@@ -24810,7 +24810,7 @@
       </c>
       <c r="N246" s="2" t="inlineStr">
         <is>
-          <t>1.042s</t>
+          <t>0.105s</t>
         </is>
       </c>
       <c r="O246" s="3" t="inlineStr">
@@ -24909,7 +24909,7 @@
       </c>
       <c r="N247" s="2" t="inlineStr">
         <is>
-          <t>1.571s</t>
+          <t>1.444s</t>
         </is>
       </c>
       <c r="O247" s="3" t="inlineStr">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="N248" s="2" t="inlineStr">
         <is>
-          <t>1.321s</t>
+          <t>1.390s</t>
         </is>
       </c>
       <c r="O248" s="3" t="inlineStr">
@@ -25107,7 +25107,7 @@
       </c>
       <c r="N249" s="2" t="inlineStr">
         <is>
-          <t>0.596s</t>
+          <t>1.534s</t>
         </is>
       </c>
       <c r="O249" s="3" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="N250" s="2" t="inlineStr">
         <is>
-          <t>0.159s</t>
+          <t>0.527s</t>
         </is>
       </c>
       <c r="O250" s="3" t="inlineStr">
@@ -25305,7 +25305,7 @@
       </c>
       <c r="N251" s="2" t="inlineStr">
         <is>
-          <t>0.907s</t>
+          <t>1.215s</t>
         </is>
       </c>
       <c r="O251" s="3" t="inlineStr">
@@ -25404,7 +25404,7 @@
       </c>
       <c r="N252" s="2" t="inlineStr">
         <is>
-          <t>0.714s</t>
+          <t>1.229s</t>
         </is>
       </c>
       <c r="O252" s="3" t="inlineStr">
@@ -25503,7 +25503,7 @@
       </c>
       <c r="N253" s="2" t="inlineStr">
         <is>
-          <t>1.338s</t>
+          <t>0.459s</t>
         </is>
       </c>
       <c r="O253" s="3" t="inlineStr">
@@ -25602,7 +25602,7 @@
       </c>
       <c r="N254" s="2" t="inlineStr">
         <is>
-          <t>0.683s</t>
+          <t>1.402s</t>
         </is>
       </c>
       <c r="O254" s="3" t="inlineStr">
@@ -25701,7 +25701,7 @@
       </c>
       <c r="N255" s="2" t="inlineStr">
         <is>
-          <t>0.258s</t>
+          <t>1.328s</t>
         </is>
       </c>
       <c r="O255" s="3" t="inlineStr">
@@ -25800,7 +25800,7 @@
       </c>
       <c r="N256" s="2" t="inlineStr">
         <is>
-          <t>0.337s</t>
+          <t>1.089s</t>
         </is>
       </c>
       <c r="O256" s="3" t="inlineStr">
@@ -25899,7 +25899,7 @@
       </c>
       <c r="N257" s="2" t="inlineStr">
         <is>
-          <t>1.602s</t>
+          <t>1.483s</t>
         </is>
       </c>
       <c r="O257" s="3" t="inlineStr">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="N258" s="2" t="inlineStr">
         <is>
-          <t>1.676s</t>
+          <t>0.355s</t>
         </is>
       </c>
       <c r="O258" s="3" t="inlineStr">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="N259" s="2" t="inlineStr">
         <is>
-          <t>1.402s</t>
+          <t>1.080s</t>
         </is>
       </c>
       <c r="O259" s="3" t="inlineStr">
@@ -26196,7 +26196,7 @@
       </c>
       <c r="N260" s="2" t="inlineStr">
         <is>
-          <t>0.802s</t>
+          <t>1.656s</t>
         </is>
       </c>
       <c r="O260" s="3" t="inlineStr">
@@ -26295,7 +26295,7 @@
       </c>
       <c r="N261" s="2" t="inlineStr">
         <is>
-          <t>1.725s</t>
+          <t>1.207s</t>
         </is>
       </c>
       <c r="O261" s="3" t="inlineStr">
@@ -26394,7 +26394,7 @@
       </c>
       <c r="N262" s="2" t="inlineStr">
         <is>
-          <t>1.651s</t>
+          <t>0.074s</t>
         </is>
       </c>
       <c r="O262" s="3" t="inlineStr">
@@ -26493,7 +26493,7 @@
       </c>
       <c r="N263" s="2" t="inlineStr">
         <is>
-          <t>1.101s</t>
+          <t>0.995s</t>
         </is>
       </c>
       <c r="O263" s="3" t="inlineStr">
@@ -26592,7 +26592,7 @@
       </c>
       <c r="N264" s="2" t="inlineStr">
         <is>
-          <t>1.803s</t>
+          <t>1.232s</t>
         </is>
       </c>
       <c r="O264" s="3" t="inlineStr">
@@ -26691,7 +26691,7 @@
       </c>
       <c r="N265" s="2" t="inlineStr">
         <is>
-          <t>1.722s</t>
+          <t>0.084s</t>
         </is>
       </c>
       <c r="O265" s="3" t="inlineStr">
@@ -26790,7 +26790,7 @@
       </c>
       <c r="N266" s="2" t="inlineStr">
         <is>
-          <t>1.132s</t>
+          <t>0.788s</t>
         </is>
       </c>
       <c r="O266" s="3" t="inlineStr">
@@ -26889,7 +26889,7 @@
       </c>
       <c r="N267" s="2" t="inlineStr">
         <is>
-          <t>0.498s</t>
+          <t>0.523s</t>
         </is>
       </c>
       <c r="O267" s="3" t="inlineStr">
@@ -26988,7 +26988,7 @@
       </c>
       <c r="N268" s="2" t="inlineStr">
         <is>
-          <t>1.053s</t>
+          <t>0.137s</t>
         </is>
       </c>
       <c r="O268" s="3" t="inlineStr">
@@ -27087,7 +27087,7 @@
       </c>
       <c r="N269" s="2" t="inlineStr">
         <is>
-          <t>1.192s</t>
+          <t>0.590s</t>
         </is>
       </c>
       <c r="O269" s="3" t="inlineStr">
@@ -27186,7 +27186,7 @@
       </c>
       <c r="N270" s="2" t="inlineStr">
         <is>
-          <t>0.496s</t>
+          <t>1.000s</t>
         </is>
       </c>
       <c r="O270" s="3" t="inlineStr">
@@ -27285,7 +27285,7 @@
       </c>
       <c r="N271" s="2" t="inlineStr">
         <is>
-          <t>0.254s</t>
+          <t>1.519s</t>
         </is>
       </c>
       <c r="O271" s="3" t="inlineStr">
@@ -27384,7 +27384,7 @@
       </c>
       <c r="N272" s="2" t="inlineStr">
         <is>
-          <t>1.357s</t>
+          <t>0.865s</t>
         </is>
       </c>
       <c r="O272" s="3" t="inlineStr">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="N273" s="2" t="inlineStr">
         <is>
-          <t>0.833s</t>
+          <t>0.072s</t>
         </is>
       </c>
       <c r="O273" s="3" t="inlineStr">
@@ -27582,7 +27582,7 @@
       </c>
       <c r="N274" s="2" t="inlineStr">
         <is>
-          <t>0.596s</t>
+          <t>1.382s</t>
         </is>
       </c>
       <c r="O274" s="3" t="inlineStr">
@@ -27681,7 +27681,7 @@
       </c>
       <c r="N275" s="2" t="inlineStr">
         <is>
-          <t>0.851s</t>
+          <t>0.578s</t>
         </is>
       </c>
       <c r="O275" s="3" t="inlineStr">
@@ -27780,7 +27780,7 @@
       </c>
       <c r="N276" s="2" t="inlineStr">
         <is>
-          <t>1.626s</t>
+          <t>0.502s</t>
         </is>
       </c>
       <c r="O276" s="3" t="inlineStr">
@@ -27879,7 +27879,7 @@
       </c>
       <c r="N277" s="2" t="inlineStr">
         <is>
-          <t>0.622s</t>
+          <t>1.325s</t>
         </is>
       </c>
       <c r="O277" s="3" t="inlineStr">
@@ -27978,7 +27978,7 @@
       </c>
       <c r="N278" s="2" t="inlineStr">
         <is>
-          <t>0.457s</t>
+          <t>0.284s</t>
         </is>
       </c>
       <c r="O278" s="3" t="inlineStr">
@@ -28077,7 +28077,7 @@
       </c>
       <c r="N279" s="2" t="inlineStr">
         <is>
-          <t>1.267s</t>
+          <t>1.474s</t>
         </is>
       </c>
       <c r="O279" s="3" t="inlineStr">
@@ -28176,7 +28176,7 @@
       </c>
       <c r="N280" s="2" t="inlineStr">
         <is>
-          <t>0.861s</t>
+          <t>0.740s</t>
         </is>
       </c>
       <c r="O280" s="3" t="inlineStr">
@@ -28275,7 +28275,7 @@
       </c>
       <c r="N281" s="2" t="inlineStr">
         <is>
-          <t>0.862s</t>
+          <t>1.809s</t>
         </is>
       </c>
       <c r="O281" s="3" t="inlineStr">
@@ -28374,7 +28374,7 @@
       </c>
       <c r="N282" s="2" t="inlineStr">
         <is>
-          <t>1.656s</t>
+          <t>1.310s</t>
         </is>
       </c>
       <c r="O282" s="3" t="inlineStr">
@@ -28473,7 +28473,7 @@
       </c>
       <c r="N283" s="2" t="inlineStr">
         <is>
-          <t>1.751s</t>
+          <t>0.481s</t>
         </is>
       </c>
       <c r="O283" s="3" t="inlineStr">
@@ -28572,7 +28572,7 @@
       </c>
       <c r="N284" s="2" t="inlineStr">
         <is>
-          <t>1.512s</t>
+          <t>1.177s</t>
         </is>
       </c>
       <c r="O284" s="3" t="inlineStr">
@@ -28671,7 +28671,7 @@
       </c>
       <c r="N285" s="2" t="inlineStr">
         <is>
-          <t>1.724s</t>
+          <t>1.778s</t>
         </is>
       </c>
       <c r="O285" s="3" t="inlineStr">
@@ -28770,7 +28770,7 @@
       </c>
       <c r="N286" s="2" t="inlineStr">
         <is>
-          <t>1.820s</t>
+          <t>1.076s</t>
         </is>
       </c>
       <c r="O286" s="3" t="inlineStr">
@@ -28869,7 +28869,7 @@
       </c>
       <c r="N287" s="2" t="inlineStr">
         <is>
-          <t>1.257s</t>
+          <t>0.296s</t>
         </is>
       </c>
       <c r="O287" s="3" t="inlineStr">
@@ -28968,7 +28968,7 @@
       </c>
       <c r="N288" s="2" t="inlineStr">
         <is>
-          <t>1.303s</t>
+          <t>1.580s</t>
         </is>
       </c>
       <c r="O288" s="3" t="inlineStr">
@@ -29067,7 +29067,7 @@
       </c>
       <c r="N289" s="2" t="inlineStr">
         <is>
-          <t>0.730s</t>
+          <t>0.867s</t>
         </is>
       </c>
       <c r="O289" s="3" t="inlineStr">
@@ -29166,7 +29166,7 @@
       </c>
       <c r="N290" s="2" t="inlineStr">
         <is>
-          <t>0.839s</t>
+          <t>1.611s</t>
         </is>
       </c>
       <c r="O290" s="3" t="inlineStr">
@@ -29265,7 +29265,7 @@
       </c>
       <c r="N291" s="2" t="inlineStr">
         <is>
-          <t>0.237s</t>
+          <t>0.780s</t>
         </is>
       </c>
       <c r="O291" s="3" t="inlineStr">
@@ -29364,7 +29364,7 @@
       </c>
       <c r="N292" s="2" t="inlineStr">
         <is>
-          <t>1.735s</t>
+          <t>1.554s</t>
         </is>
       </c>
       <c r="O292" s="3" t="inlineStr">
@@ -29463,7 +29463,7 @@
       </c>
       <c r="N293" s="2" t="inlineStr">
         <is>
-          <t>1.108s</t>
+          <t>1.477s</t>
         </is>
       </c>
       <c r="O293" s="3" t="inlineStr">
@@ -29562,7 +29562,7 @@
       </c>
       <c r="N294" s="2" t="inlineStr">
         <is>
-          <t>0.491s</t>
+          <t>1.013s</t>
         </is>
       </c>
       <c r="O294" s="3" t="inlineStr">
@@ -29661,7 +29661,7 @@
       </c>
       <c r="N295" s="2" t="inlineStr">
         <is>
-          <t>1.769s</t>
+          <t>0.854s</t>
         </is>
       </c>
       <c r="O295" s="3" t="inlineStr">
@@ -29760,7 +29760,7 @@
       </c>
       <c r="N296" s="2" t="inlineStr">
         <is>
-          <t>1.193s</t>
+          <t>1.503s</t>
         </is>
       </c>
       <c r="O296" s="3" t="inlineStr">
@@ -29859,7 +29859,7 @@
       </c>
       <c r="N297" s="2" t="inlineStr">
         <is>
-          <t>0.615s</t>
+          <t>0.558s</t>
         </is>
       </c>
       <c r="O297" s="3" t="inlineStr">
@@ -29958,7 +29958,7 @@
       </c>
       <c r="N298" s="2" t="inlineStr">
         <is>
-          <t>1.528s</t>
+          <t>0.619s</t>
         </is>
       </c>
       <c r="O298" s="3" t="inlineStr">
@@ -30057,7 +30057,7 @@
       </c>
       <c r="N299" s="2" t="inlineStr">
         <is>
-          <t>1.138s</t>
+          <t>1.353s</t>
         </is>
       </c>
       <c r="O299" s="3" t="inlineStr">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="N300" s="2" t="inlineStr">
         <is>
-          <t>0.888s</t>
+          <t>1.524s</t>
         </is>
       </c>
       <c r="O300" s="3" t="inlineStr">
@@ -30255,7 +30255,7 @@
       </c>
       <c r="N301" s="2" t="inlineStr">
         <is>
-          <t>1.379s</t>
+          <t>1.330s</t>
         </is>
       </c>
       <c r="O301" s="3" t="inlineStr">

</xml_diff>